<commit_message>
Primeiras 5 fotos reais: Trevi, Sagrada Família, Big Ben, Beihai e Zanzibar
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bcj52n14kthUhgj2yyyAud
</commit_message>
<xml_diff>
--- a/content/biblioteca-inicial.xlsx
+++ b/content/biblioteca-inicial.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1181" uniqueCount="521">
   <si>
     <t>destination_id</t>
   </si>
@@ -434,6 +434,30 @@
     <t>America/Aruba</t>
   </si>
   <si>
+    <t>tanzania</t>
+  </si>
+  <si>
+    <t>Tanzânia</t>
+  </si>
+  <si>
+    <t>Africa/Dar_es_Salaam</t>
+  </si>
+  <si>
+    <t>zanzibar</t>
+  </si>
+  <si>
+    <t>Arquipélago de Zanzibar</t>
+  </si>
+  <si>
+    <t>Zanzibar</t>
+  </si>
+  <si>
+    <t>Ilha de mar azul-piscina, areia branquinha e barcos de madeira tradicionais. As praias do norte são as mais procuradas.</t>
+  </si>
+  <si>
+    <t>Junho a outubro; dezembro a fevereiro</t>
+  </si>
+  <si>
     <t>portugal</t>
   </si>
   <si>
@@ -1022,6 +1046,21 @@
     <t>Badaling, Yanqing, Pequim, China</t>
   </si>
   <si>
+    <t>pequim-beihai</t>
+  </si>
+  <si>
+    <t>Parque Beihai</t>
+  </si>
+  <si>
+    <t>Parque imperial com lago, pavilhões vermelhos e dourados e pontes de pedra. Ótimo no fim de tarde.</t>
+  </si>
+  <si>
+    <t>1 Wenjin St, Xicheng, Pequim, China</t>
+  </si>
+  <si>
+    <t>parque, história</t>
+  </si>
+  <si>
     <t>pequim-cidade-proibida</t>
   </si>
   <si>
@@ -1443,6 +1482,21 @@
   </si>
   <si>
     <t>natureza, aventura</t>
+  </si>
+  <si>
+    <t>zanzibar-praias-norte</t>
+  </si>
+  <si>
+    <t>Praias do norte (Nungwi e Kendwa)</t>
+  </si>
+  <si>
+    <t>Areia clara, mar transparente e pôr do sol de cartão-postal. Dá pra passear de barco tradicional (dhow).</t>
+  </si>
+  <si>
+    <t>Nungwi, Zanzibar, Tanzânia</t>
+  </si>
+  <si>
+    <t>praia, pôr do sol</t>
   </si>
   <si>
     <t>lisboa-torre-de-belem</t>
@@ -1901,7 +1955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2898,19 +2952,19 @@
         <v>141</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>144</v>
       </c>
       <c r="D35" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H35" t="s">
         <v>142</v>
@@ -2921,10 +2975,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B36" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C36" t="s">
         <v>11</v>
@@ -2942,7 +2996,7 @@
         <v>11</v>
       </c>
       <c r="H36" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I36" t="s">
         <v>11</v>
@@ -2950,31 +3004,89 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>151</v>
+      </c>
+      <c r="B37" t="s">
+        <v>149</v>
+      </c>
+      <c r="C37" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" t="s">
+        <v>152</v>
+      </c>
+      <c r="E37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" t="s">
+        <v>153</v>
+      </c>
+      <c r="G37" t="s">
+        <v>154</v>
+      </c>
+      <c r="H37" t="s">
         <v>150</v>
       </c>
-      <c r="B37" t="s">
+      <c r="I37" t="s">
         <v>148</v>
       </c>
-      <c r="C37" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" t="s">
-        <v>151</v>
-      </c>
-      <c r="E37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" t="s">
-        <v>152</v>
-      </c>
-      <c r="G37" t="s">
-        <v>153</v>
-      </c>
-      <c r="H37" t="s">
-        <v>149</v>
-      </c>
-      <c r="I37" t="s">
-        <v>147</v>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>155</v>
+      </c>
+      <c r="B38" t="s">
+        <v>156</v>
+      </c>
+      <c r="C38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" t="s">
+        <v>11</v>
+      </c>
+      <c r="G38" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" t="s">
+        <v>157</v>
+      </c>
+      <c r="I38" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>158</v>
+      </c>
+      <c r="B39" t="s">
+        <v>156</v>
+      </c>
+      <c r="C39" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" t="s">
+        <v>159</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" t="s">
+        <v>160</v>
+      </c>
+      <c r="G39" t="s">
+        <v>161</v>
+      </c>
+      <c r="H39" t="s">
+        <v>157</v>
+      </c>
+      <c r="I39" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2985,71 +3097,71 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E2" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F2" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="G2">
         <v>-22.9519</v>
@@ -3061,39 +3173,39 @@
         <v>11</v>
       </c>
       <c r="J2" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="K2" t="s">
         <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M2" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N2" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D3" t="s">
         <v>177</v>
       </c>
-      <c r="D3" t="s">
-        <v>169</v>
-      </c>
       <c r="E3" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="F3" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="G3">
         <v>-22.9486</v>
@@ -3102,42 +3214,42 @@
         <v>-43.1566</v>
       </c>
       <c r="I3" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="J3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="K3" t="s">
         <v>11</v>
       </c>
       <c r="L3" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M3" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N3" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E4" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F4" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="G4">
         <v>-22.9154</v>
@@ -3149,39 +3261,39 @@
         <v>11</v>
       </c>
       <c r="J4" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="K4" t="s">
         <v>11</v>
       </c>
       <c r="L4" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M4" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N4" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F5" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="G5">
         <v>-22.9711</v>
@@ -3193,39 +3305,39 @@
         <v>11</v>
       </c>
       <c r="J5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="K5" t="s">
         <v>11</v>
       </c>
       <c r="L5" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M5" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N5" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D6" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E6" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="F6" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="G6">
         <v>-22.9668</v>
@@ -3237,39 +3349,39 @@
         <v>11</v>
       </c>
       <c r="J6" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="K6" t="s">
         <v>11</v>
       </c>
       <c r="L6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M6" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N6" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D7" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E7" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="F7" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="G7">
         <v>48.8584</v>
@@ -3278,42 +3390,42 @@
         <v>2.2945</v>
       </c>
       <c r="I7" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="J7" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="K7" t="s">
         <v>11</v>
       </c>
       <c r="L7" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M7" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N7" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D8" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E8" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F8" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="G8">
         <v>48.8606</v>
@@ -3322,42 +3434,42 @@
         <v>2.3376</v>
       </c>
       <c r="I8" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="J8" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="K8" t="s">
         <v>11</v>
       </c>
       <c r="L8" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N8" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D9" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="F9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="G9">
         <v>48.86</v>
@@ -3366,42 +3478,42 @@
         <v>2.3266</v>
       </c>
       <c r="I9" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="J9" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="K9" t="s">
         <v>11</v>
       </c>
       <c r="L9" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D10" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E10" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="F10" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="G10">
         <v>48.8738</v>
@@ -3410,42 +3522,42 @@
         <v>2.295</v>
       </c>
       <c r="I10" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="J10" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="K10" t="s">
         <v>11</v>
       </c>
       <c r="L10" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M10" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N10" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="D11" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E11" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F11" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="G11">
         <v>48.8867</v>
@@ -3457,39 +3569,39 @@
         <v>11</v>
       </c>
       <c r="J11" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="K11" t="s">
         <v>11</v>
       </c>
       <c r="L11" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M11" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N11" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B12" t="s">
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="D12" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E12" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="F12" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="G12">
         <v>51.5007</v>
@@ -3501,39 +3613,39 @@
         <v>11</v>
       </c>
       <c r="J12" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="K12" t="s">
         <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M12" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N12" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D13" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E13" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="F13" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="G13">
         <v>51.5033</v>
@@ -3542,42 +3654,42 @@
         <v>-0.1196</v>
       </c>
       <c r="I13" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="J13" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="K13" t="s">
         <v>11</v>
       </c>
       <c r="L13" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M13" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N13" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D14" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E14" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="F14" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="G14">
         <v>51.5194</v>
@@ -3586,42 +3698,42 @@
         <v>-0.127</v>
       </c>
       <c r="I14" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="J14" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="K14" t="s">
         <v>11</v>
       </c>
       <c r="L14" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M14" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N14" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D15" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E15" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F15" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="G15">
         <v>51.5081</v>
@@ -3630,42 +3742,42 @@
         <v>-0.0759</v>
       </c>
       <c r="I15" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="J15" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="K15" t="s">
         <v>11</v>
       </c>
       <c r="L15" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M15" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N15" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D16" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="E16" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="F16" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="G16">
         <v>51.5413</v>
@@ -3677,39 +3789,39 @@
         <v>11</v>
       </c>
       <c r="J16" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="K16" t="s">
         <v>11</v>
       </c>
       <c r="L16" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M16" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N16" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B17" t="s">
         <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="D17" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E17" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="F17" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="G17">
         <v>28.4177</v>
@@ -3718,42 +3830,42 @@
         <v>-81.5812</v>
       </c>
       <c r="I17" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="J17" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="K17" t="s">
         <v>11</v>
       </c>
       <c r="L17" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M17" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N17" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B18" t="s">
         <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D18" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E18" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="F18" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="G18">
         <v>28.3747</v>
@@ -3762,42 +3874,42 @@
         <v>-81.5494</v>
       </c>
       <c r="I18" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="J18" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="K18" t="s">
         <v>11</v>
       </c>
       <c r="L18" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M18" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N18" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="B19" t="s">
         <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D19" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E19" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="F19" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="G19">
         <v>28.4743</v>
@@ -3806,42 +3918,42 @@
         <v>-81.4678</v>
       </c>
       <c r="I19" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="J19" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="K19" t="s">
         <v>11</v>
       </c>
       <c r="L19" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M19" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N19" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B20" t="s">
         <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="D20" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="E20" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="F20" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="G20">
         <v>28.371</v>
@@ -3853,39 +3965,39 @@
         <v>11</v>
       </c>
       <c r="J20" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="K20" t="s">
         <v>11</v>
       </c>
       <c r="L20" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M20" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N20" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B21" t="s">
         <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="D21" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E21" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="F21" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G21">
         <v>40.6892</v>
@@ -3894,42 +4006,42 @@
         <v>-74.0445</v>
       </c>
       <c r="I21" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="J21" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="K21" t="s">
         <v>11</v>
       </c>
       <c r="L21" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M21" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N21" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="B22" t="s">
         <v>42</v>
       </c>
       <c r="C22" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="D22" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E22" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="F22" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="G22">
         <v>40.7829</v>
@@ -3938,42 +4050,42 @@
         <v>-73.9654</v>
       </c>
       <c r="I22" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="J22" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="K22" t="s">
         <v>11</v>
       </c>
       <c r="L22" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M22" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N22" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B23" t="s">
         <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D23" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E23" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="F23" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="G23">
         <v>40.7614</v>
@@ -3982,42 +4094,42 @@
         <v>-73.9776</v>
       </c>
       <c r="I23" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="J23" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="K23" t="s">
         <v>11</v>
       </c>
       <c r="L23" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M23" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N23" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B24" t="s">
         <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="D24" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E24" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="F24" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="G24">
         <v>40.758</v>
@@ -4029,39 +4141,39 @@
         <v>11</v>
       </c>
       <c r="J24" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="K24" t="s">
         <v>11</v>
       </c>
       <c r="L24" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M24" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N24" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="B25" t="s">
         <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D25" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E25" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="F25" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="G25">
         <v>-13.1631</v>
@@ -4070,42 +4182,42 @@
         <v>-72.545</v>
       </c>
       <c r="I25" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="J25" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="K25" t="s">
         <v>11</v>
       </c>
       <c r="L25" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M25" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N25" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="B26" t="s">
         <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D26" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E26" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="F26" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="G26">
         <v>-13.5167</v>
@@ -4117,39 +4229,39 @@
         <v>11</v>
       </c>
       <c r="J26" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="K26" t="s">
         <v>11</v>
       </c>
       <c r="L26" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M26" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N26" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B27" t="s">
         <v>50</v>
       </c>
       <c r="C27" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="D27" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E27" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="F27" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="G27">
         <v>-13.258</v>
@@ -4161,39 +4273,39 @@
         <v>11</v>
       </c>
       <c r="J27" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="K27" t="s">
         <v>11</v>
       </c>
       <c r="L27" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M27" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N27" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="B28" t="s">
         <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D28" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E28" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="F28" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="G28">
         <v>-27.1258</v>
@@ -4205,39 +4317,39 @@
         <v>11</v>
       </c>
       <c r="J28" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="K28" t="s">
         <v>11</v>
       </c>
       <c r="L28" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M28" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N28" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="B29" t="s">
         <v>58</v>
       </c>
       <c r="C29" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="D29" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E29" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="F29" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="G29">
         <v>-27.1225</v>
@@ -4249,39 +4361,39 @@
         <v>11</v>
       </c>
       <c r="J29" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="K29" t="s">
         <v>11</v>
       </c>
       <c r="L29" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M29" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N29" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="B30" t="s">
         <v>58</v>
       </c>
       <c r="C30" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="D30" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E30" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="F30" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="G30">
         <v>-27.0733</v>
@@ -4293,39 +4405,39 @@
         <v>11</v>
       </c>
       <c r="J30" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="K30" t="s">
         <v>11</v>
       </c>
       <c r="L30" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M30" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N30" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B31" t="s">
         <v>67</v>
       </c>
       <c r="C31" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="D31" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E31" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="F31" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="G31">
         <v>40.4319</v>
@@ -4337,39 +4449,39 @@
         <v>11</v>
       </c>
       <c r="J31" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="K31" t="s">
         <v>11</v>
       </c>
       <c r="L31" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M31" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N31" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="B32" t="s">
         <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="D32" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E32" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="F32" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="G32">
         <v>40.354</v>
@@ -4381,1559 +4493,1647 @@
         <v>11</v>
       </c>
       <c r="J32" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="K32" t="s">
         <v>11</v>
       </c>
       <c r="L32" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M32" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N32" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B33" t="s">
         <v>67</v>
       </c>
       <c r="C33" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="D33" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E33" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="F33" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="G33">
-        <v>39.9163</v>
+        <v>39.9255</v>
       </c>
       <c r="H33">
-        <v>116.3972</v>
+        <v>116.3833</v>
       </c>
       <c r="I33" t="s">
         <v>11</v>
       </c>
       <c r="J33" t="s">
-        <v>244</v>
+        <v>348</v>
       </c>
       <c r="K33" t="s">
         <v>11</v>
       </c>
       <c r="L33" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M33" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N33" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="B34" t="s">
         <v>67</v>
       </c>
       <c r="C34" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="D34" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E34" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="F34" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="G34">
-        <v>39.8822</v>
+        <v>39.9163</v>
       </c>
       <c r="H34">
-        <v>116.4066</v>
+        <v>116.3972</v>
       </c>
       <c r="I34" t="s">
         <v>11</v>
       </c>
       <c r="J34" t="s">
-        <v>344</v>
+        <v>252</v>
       </c>
       <c r="K34" t="s">
         <v>11</v>
       </c>
       <c r="L34" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M34" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N34" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B35" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C35" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D35" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E35" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="F35" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="G35">
-        <v>41.8902</v>
+        <v>39.8822</v>
       </c>
       <c r="H35">
-        <v>12.4922</v>
+        <v>116.4066</v>
       </c>
       <c r="I35" t="s">
-        <v>349</v>
+        <v>11</v>
       </c>
       <c r="J35" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="K35" t="s">
         <v>11</v>
       </c>
       <c r="L35" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M35" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N35" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B36" t="s">
         <v>74</v>
       </c>
       <c r="C36" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="D36" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E36" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="F36" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="G36">
-        <v>41.9009</v>
+        <v>41.8902</v>
       </c>
       <c r="H36">
-        <v>12.4833</v>
+        <v>12.4922</v>
       </c>
       <c r="I36" t="s">
-        <v>11</v>
+        <v>362</v>
       </c>
       <c r="J36" t="s">
-        <v>283</v>
+        <v>363</v>
       </c>
       <c r="K36" t="s">
         <v>11</v>
       </c>
       <c r="L36" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M36" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N36" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="B37" t="s">
         <v>74</v>
       </c>
       <c r="C37" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="D37" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E37" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="F37" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="G37">
-        <v>41.9065</v>
+        <v>41.9009</v>
       </c>
       <c r="H37">
-        <v>12.4536</v>
+        <v>12.4833</v>
       </c>
       <c r="I37" t="s">
-        <v>359</v>
+        <v>11</v>
       </c>
       <c r="J37" t="s">
-        <v>210</v>
+        <v>291</v>
       </c>
       <c r="K37" t="s">
         <v>11</v>
       </c>
       <c r="L37" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M37" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N37" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B38" t="s">
         <v>74</v>
       </c>
       <c r="C38" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D38" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E38" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="F38" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="G38">
-        <v>41.8986</v>
+        <v>41.9065</v>
       </c>
       <c r="H38">
-        <v>12.4769</v>
+        <v>12.4536</v>
       </c>
       <c r="I38" t="s">
-        <v>11</v>
+        <v>372</v>
       </c>
       <c r="J38" t="s">
-        <v>244</v>
+        <v>218</v>
       </c>
       <c r="K38" t="s">
         <v>11</v>
       </c>
       <c r="L38" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M38" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N38" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="B39" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C39" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="D39" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E39" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="F39" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="G39">
-        <v>43.7678</v>
+        <v>41.8986</v>
       </c>
       <c r="H39">
-        <v>11.2553</v>
+        <v>12.4769</v>
       </c>
       <c r="I39" t="s">
-        <v>368</v>
+        <v>11</v>
       </c>
       <c r="J39" t="s">
-        <v>216</v>
+        <v>252</v>
       </c>
       <c r="K39" t="s">
         <v>11</v>
       </c>
       <c r="L39" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M39" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N39" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B40" t="s">
         <v>78</v>
       </c>
       <c r="C40" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D40" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E40" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="F40" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="G40">
-        <v>43.7731</v>
+        <v>43.7678</v>
       </c>
       <c r="H40">
-        <v>11.256</v>
+        <v>11.2553</v>
       </c>
       <c r="I40" t="s">
-        <v>11</v>
+        <v>381</v>
       </c>
       <c r="J40" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="K40" t="s">
         <v>11</v>
       </c>
       <c r="L40" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M40" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N40" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
       <c r="B41" t="s">
         <v>78</v>
       </c>
       <c r="C41" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="D41" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E41" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="F41" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="G41">
-        <v>43.768</v>
+        <v>43.7731</v>
       </c>
       <c r="H41">
-        <v>11.2531</v>
+        <v>11.256</v>
       </c>
       <c r="I41" t="s">
         <v>11</v>
       </c>
       <c r="J41" t="s">
-        <v>377</v>
+        <v>211</v>
       </c>
       <c r="K41" t="s">
         <v>11</v>
       </c>
       <c r="L41" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M41" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N41" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C42" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="D42" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E42" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="F42" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="G42">
-        <v>45.4341</v>
+        <v>43.768</v>
       </c>
       <c r="H42">
-        <v>12.3388</v>
+        <v>11.2531</v>
       </c>
       <c r="I42" t="s">
         <v>11</v>
       </c>
       <c r="J42" t="s">
-        <v>283</v>
+        <v>390</v>
       </c>
       <c r="K42" t="s">
         <v>11</v>
       </c>
       <c r="L42" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M42" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N42" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
       <c r="B43" t="s">
         <v>82</v>
       </c>
       <c r="C43" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="D43" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E43" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
       <c r="F43" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
       <c r="G43">
-        <v>45.438</v>
+        <v>45.4341</v>
       </c>
       <c r="H43">
-        <v>12.3359</v>
+        <v>12.3388</v>
       </c>
       <c r="I43" t="s">
         <v>11</v>
       </c>
       <c r="J43" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="K43" t="s">
         <v>11</v>
       </c>
       <c r="L43" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M43" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N43" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C44" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="D44" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E44" t="s">
-        <v>388</v>
+        <v>397</v>
       </c>
       <c r="F44" t="s">
-        <v>389</v>
+        <v>398</v>
       </c>
       <c r="G44">
-        <v>37.9715</v>
+        <v>45.438</v>
       </c>
       <c r="H44">
-        <v>23.7257</v>
+        <v>12.3359</v>
       </c>
       <c r="I44" t="s">
         <v>11</v>
       </c>
       <c r="J44" t="s">
-        <v>350</v>
+        <v>291</v>
       </c>
       <c r="K44" t="s">
         <v>11</v>
       </c>
       <c r="L44" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M44" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N44" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>390</v>
+        <v>399</v>
       </c>
       <c r="B45" t="s">
         <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>391</v>
+        <v>400</v>
       </c>
       <c r="D45" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E45" t="s">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="F45" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="G45">
-        <v>37.9685</v>
+        <v>37.9715</v>
       </c>
       <c r="H45">
-        <v>23.7285</v>
+        <v>23.7257</v>
       </c>
       <c r="I45" t="s">
-        <v>394</v>
+        <v>11</v>
       </c>
       <c r="J45" t="s">
-        <v>244</v>
+        <v>363</v>
       </c>
       <c r="K45" t="s">
         <v>11</v>
       </c>
       <c r="L45" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M45" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N45" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C46" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="D46" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E46" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="F46" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="G46">
-        <v>36.4618</v>
+        <v>37.9685</v>
       </c>
       <c r="H46">
-        <v>25.3753</v>
+        <v>23.7285</v>
       </c>
       <c r="I46" t="s">
-        <v>11</v>
+        <v>407</v>
       </c>
       <c r="J46" t="s">
-        <v>399</v>
+        <v>252</v>
       </c>
       <c r="K46" t="s">
         <v>11</v>
       </c>
       <c r="L46" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M46" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N46" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="B47" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C47" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="D47" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E47" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="F47" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="G47">
-        <v>41.4036</v>
+        <v>36.4618</v>
       </c>
       <c r="H47">
-        <v>2.1744</v>
+        <v>25.3753</v>
       </c>
       <c r="I47" t="s">
-        <v>404</v>
+        <v>11</v>
       </c>
       <c r="J47" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="K47" t="s">
         <v>11</v>
       </c>
       <c r="L47" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M47" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N47" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B48" t="s">
         <v>101</v>
       </c>
       <c r="C48" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="D48" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E48" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="F48" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="G48">
-        <v>41.4145</v>
+        <v>41.4036</v>
       </c>
       <c r="H48">
-        <v>2.1527</v>
+        <v>2.1744</v>
       </c>
       <c r="I48" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="J48" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="K48" t="s">
         <v>11</v>
       </c>
       <c r="L48" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M48" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N48" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C49" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="D49" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E49" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="F49" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="G49">
-        <v>40.4138</v>
+        <v>41.4145</v>
       </c>
       <c r="H49">
-        <v>-3.6921</v>
+        <v>2.1527</v>
       </c>
       <c r="I49" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="J49" t="s">
-        <v>216</v>
+        <v>424</v>
       </c>
       <c r="K49" t="s">
         <v>11</v>
       </c>
       <c r="L49" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M49" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N49" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="B50" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C50" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="D50" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E50" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="F50" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="G50">
-        <v>37.1761</v>
+        <v>40.4138</v>
       </c>
       <c r="H50">
-        <v>-3.5881</v>
+        <v>-3.6921</v>
       </c>
       <c r="I50" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="J50" t="s">
-        <v>422</v>
+        <v>224</v>
       </c>
       <c r="K50" t="s">
         <v>11</v>
       </c>
       <c r="L50" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M50" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N50" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="B51" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C51" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="D51" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="E51" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="F51" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="G51">
-        <v>63.8804</v>
+        <v>37.1761</v>
       </c>
       <c r="H51">
-        <v>-22.4495</v>
+        <v>-3.5881</v>
       </c>
       <c r="I51" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="J51" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="K51" t="s">
         <v>11</v>
       </c>
       <c r="L51" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M51" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N51" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="B52" t="s">
         <v>118</v>
       </c>
       <c r="C52" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="D52" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="E52" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="F52" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G52">
-        <v>64.1417</v>
+        <v>63.8804</v>
       </c>
       <c r="H52">
-        <v>-21.9266</v>
+        <v>-22.4495</v>
       </c>
       <c r="I52" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="J52" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="K52" t="s">
         <v>11</v>
       </c>
       <c r="L52" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M52" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N52" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="B53" t="s">
         <v>118</v>
       </c>
       <c r="C53" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="D53" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E53" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="F53" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="G53">
-        <v>64.3271</v>
+        <v>64.1417</v>
       </c>
       <c r="H53">
-        <v>-20.1199</v>
+        <v>-21.9266</v>
       </c>
       <c r="I53" t="s">
-        <v>11</v>
+        <v>446</v>
       </c>
       <c r="J53" t="s">
-        <v>197</v>
+        <v>447</v>
       </c>
       <c r="K53" t="s">
         <v>11</v>
       </c>
       <c r="L53" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M53" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N53" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>439</v>
+        <v>448</v>
       </c>
       <c r="B54" t="s">
         <v>118</v>
       </c>
       <c r="C54" t="s">
-        <v>440</v>
+        <v>449</v>
       </c>
       <c r="D54" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E54" t="s">
-        <v>441</v>
+        <v>450</v>
       </c>
       <c r="F54" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="G54">
-        <v>64.0784</v>
+        <v>64.3271</v>
       </c>
       <c r="H54">
-        <v>-16.2306</v>
+        <v>-20.1199</v>
       </c>
       <c r="I54" t="s">
         <v>11</v>
       </c>
       <c r="J54" t="s">
-        <v>443</v>
+        <v>205</v>
       </c>
       <c r="K54" t="s">
         <v>11</v>
       </c>
       <c r="L54" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M54" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N54" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="B55" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C55" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="D55" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E55" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="F55" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="G55">
-        <v>19.6925</v>
+        <v>64.0784</v>
       </c>
       <c r="H55">
-        <v>-98.8438</v>
+        <v>-16.2306</v>
       </c>
       <c r="I55" t="s">
         <v>11</v>
       </c>
       <c r="J55" t="s">
-        <v>244</v>
+        <v>456</v>
       </c>
       <c r="K55" t="s">
         <v>11</v>
       </c>
       <c r="L55" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M55" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N55" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
       <c r="B56" t="s">
         <v>126</v>
       </c>
       <c r="C56" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="D56" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E56" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="F56" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
       <c r="G56">
-        <v>19.426</v>
+        <v>19.6925</v>
       </c>
       <c r="H56">
-        <v>-99.1863</v>
+        <v>-98.8438</v>
       </c>
       <c r="I56" t="s">
-        <v>452</v>
+        <v>11</v>
       </c>
       <c r="J56" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="K56" t="s">
         <v>11</v>
       </c>
       <c r="L56" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M56" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N56" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="B57" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C57" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="D57" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E57" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="F57" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="G57">
-        <v>20.6843</v>
+        <v>19.426</v>
       </c>
       <c r="H57">
-        <v>-88.5678</v>
+        <v>-99.1863</v>
       </c>
       <c r="I57" t="s">
-        <v>11</v>
+        <v>465</v>
       </c>
       <c r="J57" t="s">
-        <v>350</v>
+        <v>252</v>
       </c>
       <c r="K57" t="s">
         <v>11</v>
       </c>
       <c r="L57" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M57" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N57" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="B58" t="s">
         <v>129</v>
       </c>
       <c r="C58" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="D58" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E58" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="F58" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
       <c r="G58">
-        <v>20.2149</v>
+        <v>20.6843</v>
       </c>
       <c r="H58">
-        <v>-87.4291</v>
+        <v>-88.5678</v>
       </c>
       <c r="I58" t="s">
         <v>11</v>
       </c>
       <c r="J58" t="s">
-        <v>461</v>
+        <v>363</v>
       </c>
       <c r="K58" t="s">
         <v>11</v>
       </c>
       <c r="L58" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M58" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N58" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="B59" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C59" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="D59" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E59" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="F59" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="G59">
-        <v>12.55</v>
+        <v>20.2149</v>
       </c>
       <c r="H59">
-        <v>-70.057</v>
+        <v>-87.4291</v>
       </c>
       <c r="I59" t="s">
         <v>11</v>
       </c>
       <c r="J59" t="s">
-        <v>191</v>
+        <v>474</v>
       </c>
       <c r="K59" t="s">
         <v>11</v>
       </c>
       <c r="L59" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M59" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N59" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="B60" t="s">
         <v>135</v>
       </c>
       <c r="C60" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
       <c r="D60" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E60" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="F60" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="G60">
-        <v>12.58</v>
+        <v>12.55</v>
       </c>
       <c r="H60">
-        <v>-70.045</v>
+        <v>-70.057</v>
       </c>
       <c r="I60" t="s">
         <v>11</v>
       </c>
       <c r="J60" t="s">
-        <v>470</v>
+        <v>199</v>
       </c>
       <c r="K60" t="s">
         <v>11</v>
       </c>
       <c r="L60" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M60" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N60" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="B61" t="s">
         <v>135</v>
       </c>
       <c r="C61" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="D61" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="E61" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="F61" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="G61">
-        <v>12.495</v>
+        <v>12.58</v>
       </c>
       <c r="H61">
-        <v>-69.945</v>
+        <v>-70.045</v>
       </c>
       <c r="I61" t="s">
-        <v>475</v>
+        <v>11</v>
       </c>
       <c r="J61" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="K61" t="s">
         <v>11</v>
       </c>
       <c r="L61" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M61" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N61" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="B62" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C62" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="D62" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="E62" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="F62" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="G62">
-        <v>38.6916</v>
+        <v>12.495</v>
       </c>
       <c r="H62">
-        <v>-9.216</v>
+        <v>-69.945</v>
       </c>
       <c r="I62" t="s">
-        <v>11</v>
+        <v>488</v>
       </c>
       <c r="J62" t="s">
-        <v>350</v>
+        <v>489</v>
       </c>
       <c r="K62" t="s">
         <v>11</v>
       </c>
       <c r="L62" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M62" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N62" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="B63" t="s">
         <v>143</v>
       </c>
       <c r="C63" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="D63" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="E63" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="F63" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="G63">
-        <v>38.6979</v>
+        <v>-5.7256</v>
       </c>
       <c r="H63">
-        <v>-9.2068</v>
+        <v>39.2979</v>
       </c>
       <c r="I63" t="s">
         <v>11</v>
       </c>
       <c r="J63" t="s">
-        <v>244</v>
+        <v>494</v>
       </c>
       <c r="K63" t="s">
         <v>11</v>
       </c>
       <c r="L63" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M63" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N63" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
       <c r="B64" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C64" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="D64" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="E64" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="F64" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="G64">
-        <v>38.7114</v>
+        <v>38.6916</v>
       </c>
       <c r="H64">
-        <v>-9.13</v>
+        <v>-9.216</v>
       </c>
       <c r="I64" t="s">
         <v>11</v>
       </c>
       <c r="J64" t="s">
-        <v>489</v>
+        <v>363</v>
       </c>
       <c r="K64" t="s">
         <v>11</v>
       </c>
       <c r="L64" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M64" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N64" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="B65" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C65" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="D65" t="s">
-        <v>169</v>
+        <v>214</v>
       </c>
       <c r="E65" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="F65" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="G65">
-        <v>35.7148</v>
+        <v>38.6979</v>
       </c>
       <c r="H65">
-        <v>139.7967</v>
+        <v>-9.2068</v>
       </c>
       <c r="I65" t="s">
         <v>11</v>
       </c>
       <c r="J65" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="K65" t="s">
         <v>11</v>
       </c>
       <c r="L65" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M65" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N65" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C66" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="D66" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="E66" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="F66" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="G66">
-        <v>35.6595</v>
+        <v>38.7114</v>
       </c>
       <c r="H66">
-        <v>139.7005</v>
+        <v>-9.13</v>
       </c>
       <c r="I66" t="s">
         <v>11</v>
       </c>
       <c r="J66" t="s">
-        <v>299</v>
+        <v>507</v>
       </c>
       <c r="K66" t="s">
         <v>11</v>
       </c>
       <c r="L66" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="M66" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="N66" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="B67" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C67" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="D67" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E67" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="F67" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="G67">
+        <v>35.7148</v>
+      </c>
+      <c r="H67">
+        <v>139.7967</v>
+      </c>
+      <c r="I67" t="s">
+        <v>11</v>
+      </c>
+      <c r="J67" t="s">
+        <v>252</v>
+      </c>
+      <c r="K67" t="s">
+        <v>11</v>
+      </c>
+      <c r="L67" t="s">
+        <v>181</v>
+      </c>
+      <c r="M67" t="s">
+        <v>182</v>
+      </c>
+      <c r="N67" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>512</v>
+      </c>
+      <c r="B68" t="s">
+        <v>158</v>
+      </c>
+      <c r="C68" t="s">
+        <v>513</v>
+      </c>
+      <c r="D68" t="s">
+        <v>177</v>
+      </c>
+      <c r="E68" t="s">
+        <v>514</v>
+      </c>
+      <c r="F68" t="s">
+        <v>515</v>
+      </c>
+      <c r="G68">
+        <v>35.6595</v>
+      </c>
+      <c r="H68">
+        <v>139.7005</v>
+      </c>
+      <c r="I68" t="s">
+        <v>11</v>
+      </c>
+      <c r="J68" t="s">
+        <v>307</v>
+      </c>
+      <c r="K68" t="s">
+        <v>11</v>
+      </c>
+      <c r="L68" t="s">
+        <v>181</v>
+      </c>
+      <c r="M68" t="s">
+        <v>182</v>
+      </c>
+      <c r="N68" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>516</v>
+      </c>
+      <c r="B69" t="s">
+        <v>158</v>
+      </c>
+      <c r="C69" t="s">
+        <v>517</v>
+      </c>
+      <c r="D69" t="s">
+        <v>177</v>
+      </c>
+      <c r="E69" t="s">
+        <v>518</v>
+      </c>
+      <c r="F69" t="s">
+        <v>519</v>
+      </c>
+      <c r="G69">
         <v>35.7101</v>
       </c>
-      <c r="H67">
+      <c r="H69">
         <v>139.8107</v>
       </c>
-      <c r="I67" t="s">
-        <v>502</v>
-      </c>
-      <c r="J67" t="s">
-        <v>238</v>
-      </c>
-      <c r="K67" t="s">
-        <v>11</v>
-      </c>
-      <c r="L67" t="s">
-        <v>173</v>
-      </c>
-      <c r="M67" t="s">
-        <v>174</v>
-      </c>
-      <c r="N67" t="s">
-        <v>175</v>
+      <c r="I69" t="s">
+        <v>520</v>
+      </c>
+      <c r="J69" t="s">
+        <v>246</v>
+      </c>
+      <c r="K69" t="s">
+        <v>11</v>
+      </c>
+      <c r="L69" t="s">
+        <v>181</v>
+      </c>
+      <c r="M69" t="s">
+        <v>182</v>
+      </c>
+      <c r="N69" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>